<commit_message>
Ajusta mão de obra terceirizada e alinha cenários ao modo de cálculo
A obra é toda terceirizada: a parcela de mão de obra passa a ser serviço de
construção com crédito à alíquota reduzida. As colunas de cenário passam a
seguir o modo selecionado (plena ou transição), e a coluna Ativo volta a
coincidir com o cenário escolhido.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VNUG9G5PiaxGmiV8dk6CnD
</commit_message>
<xml_diff>
--- a/simulador-reforma-imoveis/simulador_reforma_tributaria_imoveis_v4.xlsx
+++ b/simulador-reforma-imoveis/simulador_reforma_tributaria_imoveis_v4.xlsx
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Resumo Executivo'!$B$1:$J$53</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Premissas &amp; Cenários'!$A$1:$I$82</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Fluxo_Incorporacao'!$A$1:$S$113</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Fluxo_Incorporacao'!$A$1:$V$113</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'DRE Empreendimento'!$A$1:$G$72</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'IRPJ_CSLL Trimestral'!$A$1:$N$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Comparativo RET'!$A$1:$H$31</definedName>
@@ -706,11 +706,11 @@
     <xf numFmtId="10" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="22" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -6339,10 +6339,9 @@
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Comparação de cenários (alíquota plena — regime de 2033 em diante)</t>
-        </is>
+      <c r="B19" s="8">
+        <f>"Comparação de cenários — modo: "&amp;'Matriz Normativa &amp; Governança'!$C$8</f>
+        <v/>
       </c>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="9" t="n"/>
@@ -6564,7 +6563,7 @@
     <row r="34" ht="63.75" customHeight="1">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Crédito de obra por composição do custo (folha sem crédito, materiais 27%, serviços de construção 13,5%) e crédito de despesas por categoria; valores com tributo embutido e cálculo por fora.</t>
+          <t>Crédito de obra por composição do custo (materiais a 27% e serviços de construção terceirizados a 13,5%; folha própria de obra, se houver, sem crédito) e crédito de despesas por categoria; valores com tributo embutido e cálculo por fora.</t>
         </is>
       </c>
     </row>
@@ -6819,7 +6818,7 @@
         <f>ROUND(B8-'Premissas &amp; Cenários'!$E$102,2)</f>
         <v/>
       </c>
-      <c r="D9" s="121" t="inlineStr">
+      <c r="D9" s="119" t="inlineStr">
         <is>
           <t>Categorias de obra: Materiais, Serviços de construção ou Mão de obra própria.</t>
         </is>
@@ -10703,15 +10702,15 @@
         </is>
       </c>
       <c r="B68" s="35">
-        <f>B67*$B$35/(1+$B$35)</f>
+        <f>IFERROR(B67/B60,0)*Fluxo_Incorporacao!$T$103</f>
         <v/>
       </c>
       <c r="C68" s="35">
-        <f>C67*$B$35/(1+$B$35)</f>
+        <f>IFERROR(C67/C60,0)*Fluxo_Incorporacao!$T$103</f>
         <v/>
       </c>
       <c r="D68" s="35">
-        <f>D67*$B$35/(1+$B$35)</f>
+        <f>IFERROR(D67/D60,0)*Fluxo_Incorporacao!$T$103</f>
         <v/>
       </c>
       <c r="F68" s="19" t="inlineStr">
@@ -10736,15 +10735,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>B58*B64</f>
+        <f>B58*B64*IFERROR(Fluxo_Incorporacao!$U$103/Fluxo_Incorporacao!$E$103,0)</f>
         <v/>
       </c>
       <c r="C69" s="33">
-        <f>C58*C64</f>
+        <f>C58*C64*IFERROR(Fluxo_Incorporacao!$U$103/Fluxo_Incorporacao!$E$103,0)</f>
         <v/>
       </c>
       <c r="D69" s="33">
-        <f>D58*D64</f>
+        <f>D58*D64*IFERROR(Fluxo_Incorporacao!$U$103/Fluxo_Incorporacao!$E$103,0)</f>
         <v/>
       </c>
       <c r="F69" s="19" t="inlineStr">
@@ -10802,15 +10801,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>$B$22*B70</f>
+        <f>$B$22*B70*IFERROR(Fluxo_Incorporacao!$V$103/Fluxo_Incorporacao!$G$103,0)</f>
         <v/>
       </c>
       <c r="C71" s="33">
-        <f>$B$22*C70</f>
+        <f>$B$22*C70*IFERROR(Fluxo_Incorporacao!$V$103/Fluxo_Incorporacao!$G$103,0)</f>
         <v/>
       </c>
       <c r="D71" s="33">
-        <f>$B$22*D70</f>
+        <f>$B$22*D70*IFERROR(Fluxo_Incorporacao!$V$103/Fluxo_Incorporacao!$G$103,0)</f>
         <v/>
       </c>
       <c r="F71" s="19" t="inlineStr">
@@ -10824,7 +10823,7 @@
       </c>
       <c r="H71" s="112" t="inlineStr">
         <is>
-          <t>Base final × alíquota efetiva ÷ (1 + alíquota): tributo embutido no preço.</t>
+          <t>Débito no modo de cálculo selecionado (plena ou transição), com tributo embutido no preço.</t>
         </is>
       </c>
     </row>
@@ -10857,7 +10856,7 @@
       </c>
       <c r="H72" s="112" t="inlineStr">
         <is>
-          <t>Custo de obra multiplicado pela média de crédito.</t>
+          <t>Custo de obra × média de crédito, na alíquota do modo de cálculo.</t>
         </is>
       </c>
     </row>
@@ -10890,7 +10889,7 @@
       </c>
       <c r="H73" s="112" t="inlineStr">
         <is>
-          <t>Créditos de obra mais despesas.</t>
+          <t>Créditos de obra mais despesas, no modo de cálculo selecionado.</t>
         </is>
       </c>
     </row>
@@ -10943,7 +10942,12 @@
         </is>
       </c>
     </row>
-    <row r="76"/>
+    <row r="76">
+      <c r="A76" s="119">
+        <f>"Os cenários seguem o modo de cálculo selecionado na Matriz: "&amp;'Matriz Normativa &amp; Governança'!$C$8</f>
+        <v/>
+      </c>
+    </row>
     <row r="77"/>
     <row r="78" ht="15" customHeight="1">
       <c r="B78" s="8" t="inlineStr">
@@ -10978,21 +10982,21 @@
     <row r="83"/>
     <row r="84"/>
     <row r="85">
-      <c r="A85" s="119" t="inlineStr">
+      <c r="A85" s="120" t="inlineStr">
         <is>
           <t>Premissas v4 — convenção de preços, composição de custos e regimes</t>
         </is>
       </c>
-      <c r="B85" s="120" t="n"/>
-      <c r="C85" s="120" t="n"/>
-      <c r="D85" s="120" t="n"/>
-      <c r="E85" s="120" t="n"/>
-      <c r="F85" s="120" t="n"/>
-      <c r="G85" s="120" t="n"/>
-      <c r="H85" s="120" t="n"/>
+      <c r="B85" s="121" t="n"/>
+      <c r="C85" s="121" t="n"/>
+      <c r="D85" s="121" t="n"/>
+      <c r="E85" s="121" t="n"/>
+      <c r="F85" s="121" t="n"/>
+      <c r="G85" s="121" t="n"/>
+      <c r="H85" s="121" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="121" t="inlineStr">
+      <c r="A86" s="119" t="inlineStr">
         <is>
           <t>Convenção: VGV, custos e despesas são informados pelo valor final pago, com IBS/CBS embutidos. Débitos e créditos são calculados por fora: tributo = valor × a ÷ (1 + a), pois o IBS/CBS não integra a própria base.</t>
         </is>
@@ -11009,15 +11013,15 @@
     <row r="89">
       <c r="A89" s="123" t="inlineStr">
         <is>
-          <t>Mão de obra própria (folha e encargos) — sem crédito</t>
+          <t>Mão de obra própria da obra (folha e encargos) — sem crédito</t>
         </is>
       </c>
       <c r="B89" s="124" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="F89" s="121" t="inlineStr">
-        <is>
-          <t>Premissa ilustrativa: substituir pela curva ABC do orçamento da obra.</t>
+        <v>0</v>
+      </c>
+      <c r="F89" s="119" t="inlineStr">
+        <is>
+          <t>Obra 100% terceirizada; a folha administrativa já está na DRE (Administração central).</t>
         </is>
       </c>
     </row>
@@ -11030,7 +11034,7 @@
       <c r="B90" s="124" t="n">
         <v>0.45</v>
       </c>
-      <c r="F90" s="121" t="inlineStr">
+      <c r="F90" s="119" t="inlineStr">
         <is>
           <t>Premissa ilustrativa: substituir pela curva ABC do orçamento da obra.</t>
         </is>
@@ -11039,13 +11043,13 @@
     <row r="91">
       <c r="A91" s="123" t="inlineStr">
         <is>
-          <t>Serviços de construção subcontratados — crédito à alíquota reduzida (art. 261)</t>
+          <t>Serviços de construção e mão de obra terceirizados — crédito à alíquota reduzida (art. 261)</t>
         </is>
       </c>
       <c r="B91" s="124" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F91" s="121" t="inlineStr">
+        <v>0.55</v>
+      </c>
+      <c r="F91" s="119" t="inlineStr">
         <is>
           <t>Premissa ilustrativa: substituir pela curva ABC do orçamento da obra.</t>
         </is>
@@ -11072,7 +11076,7 @@
         <f>B40*(1-B34)</f>
         <v/>
       </c>
-      <c r="F93" s="121" t="inlineStr">
+      <c r="F93" s="119" t="inlineStr">
         <is>
           <t>Serviço de construção também tem a redução de 50% do art. 261.</t>
         </is>
@@ -11139,7 +11143,7 @@
         <f>B97*D97*C97/(1+C97)</f>
         <v/>
       </c>
-      <c r="F97" s="121" t="inlineStr">
+      <c r="F97" s="119" t="inlineStr">
         <is>
           <t>Profissão intelectual regulamentada: redução de 30% (art. 127).</t>
         </is>
@@ -11166,7 +11170,7 @@
         <f>B98*D98*C98/(1+C98)</f>
         <v/>
       </c>
-      <c r="F98" s="121" t="inlineStr">
+      <c r="F98" s="119" t="inlineStr">
         <is>
           <t>Parte da verba vai para fornecedores do Simples ou pessoa física.</t>
         </is>
@@ -11193,7 +11197,7 @@
         <f>B99*D99*C99/(1+C99)</f>
         <v/>
       </c>
-      <c r="F99" s="121" t="inlineStr">
+      <c r="F99" s="119" t="inlineStr">
         <is>
           <t>Intermediação imobiliária: redução de 50% (art. 261); muitos corretores são PF ou Simples.</t>
         </is>
@@ -11220,7 +11224,7 @@
         <f>B100*D100*C100/(1+C100)</f>
         <v/>
       </c>
-      <c r="F100" s="121" t="inlineStr">
+      <c r="F100" s="119" t="inlineStr">
         <is>
           <t>Predominantemente folha de pagamento, que não gera crédito.</t>
         </is>
@@ -11247,7 +11251,7 @@
         <f>B101*D101*C101/(1+C101)</f>
         <v/>
       </c>
-      <c r="F101" s="121" t="inlineStr">
+      <c r="F101" s="119" t="inlineStr">
         <is>
           <t>Advocacia com redução de 30%; validar incidência sobre emolumentos.</t>
         </is>
@@ -11287,7 +11291,7 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="F105" s="121" t="inlineStr">
+      <c r="F105" s="119" t="inlineStr">
         <is>
           <t>Há liminares de TRFs suspendendo a majoração; use 'Não' para simular o cenário judicial.</t>
         </is>
@@ -11302,7 +11306,7 @@
       <c r="B106" s="131" t="n">
         <v>5000000</v>
       </c>
-      <c r="F106" s="121" t="inlineStr">
+      <c r="F106" s="119" t="inlineStr">
         <is>
           <t>Proporcional: R$ 1,25 mi por trimestre, com saldo acumulado no ano.</t>
         </is>
@@ -11317,7 +11321,7 @@
       <c r="B107" s="124" t="n">
         <v>0.1</v>
       </c>
-      <c r="F107" s="121" t="inlineStr">
+      <c r="F107" s="119" t="inlineStr">
         <is>
           <t>8% passa a 8,8% e 12% passa a 13,2% sobre o excedente.</t>
         </is>
@@ -11332,7 +11336,7 @@
       <c r="B108" s="124" t="n">
         <v>0.08799999999999999</v>
       </c>
-      <c r="F108" s="121" t="inlineStr">
+      <c r="F108" s="119" t="inlineStr">
         <is>
           <t>Estimativa; atualizar quando a alíquota de referência for fixada.</t>
         </is>
@@ -11348,7 +11352,7 @@
         <f>B33-B108</f>
         <v/>
       </c>
-      <c r="F109" s="121" t="inlineStr">
+      <c r="F109" s="119" t="inlineStr">
         <is>
           <t>Alíquota combinada menos a CBS.</t>
         </is>
@@ -11363,7 +11367,7 @@
       <c r="B110" s="132" t="n">
         <v>0.0365</v>
       </c>
-      <c r="F110" s="121" t="inlineStr">
+      <c r="F110" s="119" t="inlineStr">
         <is>
           <t>Lucro Presumido: 0,65% + 3,00% sobre a receita recebida.</t>
         </is>
@@ -11380,7 +11384,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="F111" s="121" t="inlineStr">
+      <c r="F111" s="119" t="inlineStr">
         <is>
           <t>Art. 485: 1% total (0,47% IRPJ/CSLL + 0,53% IBS/CBS).</t>
         </is>
@@ -11396,7 +11400,7 @@
         <f>IF(B111="Sim",0.01,0.04)</f>
         <v/>
       </c>
-      <c r="F112" s="121" t="inlineStr">
+      <c r="F112" s="119" t="inlineStr">
         <is>
           <t>Sobre a receita mensal recebida; sem apropriação de créditos.</t>
         </is>
@@ -11412,7 +11416,7 @@
         <f>IF(B111="Sim",0.0047,0.0192)</f>
         <v/>
       </c>
-      <c r="F113" s="121" t="inlineStr">
+      <c r="F113" s="119" t="inlineStr">
         <is>
           <t>Mesma parcela antes e depois de 2027.</t>
         </is>
@@ -11428,7 +11432,7 @@
         <f>B112-B113</f>
         <v/>
       </c>
-      <c r="F114" s="121" t="inlineStr">
+      <c r="F114" s="119" t="inlineStr">
         <is>
           <t>Art. 485: 2,08% (ou 0,53%) para opção pelo RET efetivada antes de 01/01/2029.</t>
         </is>
@@ -11443,7 +11447,7 @@
       <c r="B115" s="124" t="n">
         <v>0.12</v>
       </c>
-      <c r="F115" s="121" t="inlineStr">
+      <c r="F115" s="119" t="inlineStr">
         <is>
           <t>Usada só no comparativo de regimes.</t>
         </is>
@@ -11479,7 +11483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S113"/>
+  <dimension ref="A1:V113"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="21.140625" customWidth="1" min="1" max="1"/>
@@ -11500,6 +11504,9 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -12009,6 +12016,21 @@
           <t>Trimestre</t>
         </is>
       </c>
+      <c r="T42" s="18" t="inlineStr">
+        <is>
+          <t>Débito por R$ recebido</t>
+        </is>
+      </c>
+      <c r="U42" s="18" t="inlineStr">
+        <is>
+          <t>Obra × fator de crédito</t>
+        </is>
+      </c>
+      <c r="V42" s="18" t="inlineStr">
+        <is>
+          <t>Despesas × fator de crédito</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="31" t="n">
@@ -12086,6 +12108,18 @@
         <f>ROUNDUP(A43/3,0)</f>
         <v/>
       </c>
+      <c r="T43" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B43*$C$17/(1+$C$17),IF(O43="",0,B43*O43/(1+O43)))</f>
+        <v/>
+      </c>
+      <c r="U43" s="33">
+        <f>E43*Q43</f>
+        <v/>
+      </c>
+      <c r="V43" s="33">
+        <f>G43*Q43</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="31" t="n">
@@ -12163,6 +12197,18 @@
         <f>ROUNDUP(A44/3,0)</f>
         <v/>
       </c>
+      <c r="T44" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B44*$C$17/(1+$C$17),IF(O44="",0,B44*O44/(1+O44)))</f>
+        <v/>
+      </c>
+      <c r="U44" s="33">
+        <f>E44*Q44</f>
+        <v/>
+      </c>
+      <c r="V44" s="33">
+        <f>G44*Q44</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="31" t="n">
@@ -12240,6 +12286,18 @@
         <f>ROUNDUP(A45/3,0)</f>
         <v/>
       </c>
+      <c r="T45" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B45*$C$17/(1+$C$17),IF(O45="",0,B45*O45/(1+O45)))</f>
+        <v/>
+      </c>
+      <c r="U45" s="33">
+        <f>E45*Q45</f>
+        <v/>
+      </c>
+      <c r="V45" s="33">
+        <f>G45*Q45</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="31" t="n">
@@ -12317,6 +12375,18 @@
         <f>ROUNDUP(A46/3,0)</f>
         <v/>
       </c>
+      <c r="T46" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B46*$C$17/(1+$C$17),IF(O46="",0,B46*O46/(1+O46)))</f>
+        <v/>
+      </c>
+      <c r="U46" s="33">
+        <f>E46*Q46</f>
+        <v/>
+      </c>
+      <c r="V46" s="33">
+        <f>G46*Q46</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="31" t="n">
@@ -12394,6 +12464,18 @@
         <f>ROUNDUP(A47/3,0)</f>
         <v/>
       </c>
+      <c r="T47" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B47*$C$17/(1+$C$17),IF(O47="",0,B47*O47/(1+O47)))</f>
+        <v/>
+      </c>
+      <c r="U47" s="33">
+        <f>E47*Q47</f>
+        <v/>
+      </c>
+      <c r="V47" s="33">
+        <f>G47*Q47</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="31" t="n">
@@ -12471,6 +12553,18 @@
         <f>ROUNDUP(A48/3,0)</f>
         <v/>
       </c>
+      <c r="T48" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B48*$C$17/(1+$C$17),IF(O48="",0,B48*O48/(1+O48)))</f>
+        <v/>
+      </c>
+      <c r="U48" s="33">
+        <f>E48*Q48</f>
+        <v/>
+      </c>
+      <c r="V48" s="33">
+        <f>G48*Q48</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="31" t="n">
@@ -12548,6 +12642,18 @@
         <f>ROUNDUP(A49/3,0)</f>
         <v/>
       </c>
+      <c r="T49" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B49*$C$17/(1+$C$17),IF(O49="",0,B49*O49/(1+O49)))</f>
+        <v/>
+      </c>
+      <c r="U49" s="33">
+        <f>E49*Q49</f>
+        <v/>
+      </c>
+      <c r="V49" s="33">
+        <f>G49*Q49</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="31" t="n">
@@ -12625,6 +12731,18 @@
         <f>ROUNDUP(A50/3,0)</f>
         <v/>
       </c>
+      <c r="T50" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B50*$C$17/(1+$C$17),IF(O50="",0,B50*O50/(1+O50)))</f>
+        <v/>
+      </c>
+      <c r="U50" s="33">
+        <f>E50*Q50</f>
+        <v/>
+      </c>
+      <c r="V50" s="33">
+        <f>G50*Q50</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="31" t="n">
@@ -12702,6 +12820,18 @@
         <f>ROUNDUP(A51/3,0)</f>
         <v/>
       </c>
+      <c r="T51" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B51*$C$17/(1+$C$17),IF(O51="",0,B51*O51/(1+O51)))</f>
+        <v/>
+      </c>
+      <c r="U51" s="33">
+        <f>E51*Q51</f>
+        <v/>
+      </c>
+      <c r="V51" s="33">
+        <f>G51*Q51</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="31" t="n">
@@ -12779,6 +12909,18 @@
         <f>ROUNDUP(A52/3,0)</f>
         <v/>
       </c>
+      <c r="T52" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B52*$C$17/(1+$C$17),IF(O52="",0,B52*O52/(1+O52)))</f>
+        <v/>
+      </c>
+      <c r="U52" s="33">
+        <f>E52*Q52</f>
+        <v/>
+      </c>
+      <c r="V52" s="33">
+        <f>G52*Q52</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="31" t="n">
@@ -12856,6 +12998,18 @@
         <f>ROUNDUP(A53/3,0)</f>
         <v/>
       </c>
+      <c r="T53" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B53*$C$17/(1+$C$17),IF(O53="",0,B53*O53/(1+O53)))</f>
+        <v/>
+      </c>
+      <c r="U53" s="33">
+        <f>E53*Q53</f>
+        <v/>
+      </c>
+      <c r="V53" s="33">
+        <f>G53*Q53</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="31" t="n">
@@ -12933,6 +13087,18 @@
         <f>ROUNDUP(A54/3,0)</f>
         <v/>
       </c>
+      <c r="T54" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B54*$C$17/(1+$C$17),IF(O54="",0,B54*O54/(1+O54)))</f>
+        <v/>
+      </c>
+      <c r="U54" s="33">
+        <f>E54*Q54</f>
+        <v/>
+      </c>
+      <c r="V54" s="33">
+        <f>G54*Q54</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="31" t="n">
@@ -13010,6 +13176,18 @@
         <f>ROUNDUP(A55/3,0)</f>
         <v/>
       </c>
+      <c r="T55" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B55*$C$17/(1+$C$17),IF(O55="",0,B55*O55/(1+O55)))</f>
+        <v/>
+      </c>
+      <c r="U55" s="33">
+        <f>E55*Q55</f>
+        <v/>
+      </c>
+      <c r="V55" s="33">
+        <f>G55*Q55</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="31" t="n">
@@ -13087,6 +13265,18 @@
         <f>ROUNDUP(A56/3,0)</f>
         <v/>
       </c>
+      <c r="T56" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B56*$C$17/(1+$C$17),IF(O56="",0,B56*O56/(1+O56)))</f>
+        <v/>
+      </c>
+      <c r="U56" s="33">
+        <f>E56*Q56</f>
+        <v/>
+      </c>
+      <c r="V56" s="33">
+        <f>G56*Q56</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="31" t="n">
@@ -13164,6 +13354,18 @@
         <f>ROUNDUP(A57/3,0)</f>
         <v/>
       </c>
+      <c r="T57" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B57*$C$17/(1+$C$17),IF(O57="",0,B57*O57/(1+O57)))</f>
+        <v/>
+      </c>
+      <c r="U57" s="33">
+        <f>E57*Q57</f>
+        <v/>
+      </c>
+      <c r="V57" s="33">
+        <f>G57*Q57</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="31" t="n">
@@ -13241,6 +13443,18 @@
         <f>ROUNDUP(A58/3,0)</f>
         <v/>
       </c>
+      <c r="T58" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B58*$C$17/(1+$C$17),IF(O58="",0,B58*O58/(1+O58)))</f>
+        <v/>
+      </c>
+      <c r="U58" s="33">
+        <f>E58*Q58</f>
+        <v/>
+      </c>
+      <c r="V58" s="33">
+        <f>G58*Q58</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="31" t="n">
@@ -13318,6 +13532,18 @@
         <f>ROUNDUP(A59/3,0)</f>
         <v/>
       </c>
+      <c r="T59" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B59*$C$17/(1+$C$17),IF(O59="",0,B59*O59/(1+O59)))</f>
+        <v/>
+      </c>
+      <c r="U59" s="33">
+        <f>E59*Q59</f>
+        <v/>
+      </c>
+      <c r="V59" s="33">
+        <f>G59*Q59</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="31" t="n">
@@ -13395,6 +13621,18 @@
         <f>ROUNDUP(A60/3,0)</f>
         <v/>
       </c>
+      <c r="T60" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B60*$C$17/(1+$C$17),IF(O60="",0,B60*O60/(1+O60)))</f>
+        <v/>
+      </c>
+      <c r="U60" s="33">
+        <f>E60*Q60</f>
+        <v/>
+      </c>
+      <c r="V60" s="33">
+        <f>G60*Q60</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="31" t="n">
@@ -13472,6 +13710,18 @@
         <f>ROUNDUP(A61/3,0)</f>
         <v/>
       </c>
+      <c r="T61" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B61*$C$17/(1+$C$17),IF(O61="",0,B61*O61/(1+O61)))</f>
+        <v/>
+      </c>
+      <c r="U61" s="33">
+        <f>E61*Q61</f>
+        <v/>
+      </c>
+      <c r="V61" s="33">
+        <f>G61*Q61</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="31" t="n">
@@ -13549,6 +13799,18 @@
         <f>ROUNDUP(A62/3,0)</f>
         <v/>
       </c>
+      <c r="T62" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B62*$C$17/(1+$C$17),IF(O62="",0,B62*O62/(1+O62)))</f>
+        <v/>
+      </c>
+      <c r="U62" s="33">
+        <f>E62*Q62</f>
+        <v/>
+      </c>
+      <c r="V62" s="33">
+        <f>G62*Q62</f>
+        <v/>
+      </c>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="31" t="n">
@@ -13626,6 +13888,18 @@
         <f>ROUNDUP(A63/3,0)</f>
         <v/>
       </c>
+      <c r="T63" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B63*$C$17/(1+$C$17),IF(O63="",0,B63*O63/(1+O63)))</f>
+        <v/>
+      </c>
+      <c r="U63" s="33">
+        <f>E63*Q63</f>
+        <v/>
+      </c>
+      <c r="V63" s="33">
+        <f>G63*Q63</f>
+        <v/>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="31" t="n">
@@ -13703,6 +13977,18 @@
         <f>ROUNDUP(A64/3,0)</f>
         <v/>
       </c>
+      <c r="T64" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B64*$C$17/(1+$C$17),IF(O64="",0,B64*O64/(1+O64)))</f>
+        <v/>
+      </c>
+      <c r="U64" s="33">
+        <f>E64*Q64</f>
+        <v/>
+      </c>
+      <c r="V64" s="33">
+        <f>G64*Q64</f>
+        <v/>
+      </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="31" t="n">
@@ -13780,6 +14066,18 @@
         <f>ROUNDUP(A65/3,0)</f>
         <v/>
       </c>
+      <c r="T65" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B65*$C$17/(1+$C$17),IF(O65="",0,B65*O65/(1+O65)))</f>
+        <v/>
+      </c>
+      <c r="U65" s="33">
+        <f>E65*Q65</f>
+        <v/>
+      </c>
+      <c r="V65" s="33">
+        <f>G65*Q65</f>
+        <v/>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="31" t="n">
@@ -13857,6 +14155,18 @@
         <f>ROUNDUP(A66/3,0)</f>
         <v/>
       </c>
+      <c r="T66" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B66*$C$17/(1+$C$17),IF(O66="",0,B66*O66/(1+O66)))</f>
+        <v/>
+      </c>
+      <c r="U66" s="33">
+        <f>E66*Q66</f>
+        <v/>
+      </c>
+      <c r="V66" s="33">
+        <f>G66*Q66</f>
+        <v/>
+      </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="31" t="n">
@@ -13934,6 +14244,18 @@
         <f>ROUNDUP(A67/3,0)</f>
         <v/>
       </c>
+      <c r="T67" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B67*$C$17/(1+$C$17),IF(O67="",0,B67*O67/(1+O67)))</f>
+        <v/>
+      </c>
+      <c r="U67" s="33">
+        <f>E67*Q67</f>
+        <v/>
+      </c>
+      <c r="V67" s="33">
+        <f>G67*Q67</f>
+        <v/>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="31" t="n">
@@ -14011,6 +14333,18 @@
         <f>ROUNDUP(A68/3,0)</f>
         <v/>
       </c>
+      <c r="T68" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B68*$C$17/(1+$C$17),IF(O68="",0,B68*O68/(1+O68)))</f>
+        <v/>
+      </c>
+      <c r="U68" s="33">
+        <f>E68*Q68</f>
+        <v/>
+      </c>
+      <c r="V68" s="33">
+        <f>G68*Q68</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="31" t="n">
@@ -14088,6 +14422,18 @@
         <f>ROUNDUP(A69/3,0)</f>
         <v/>
       </c>
+      <c r="T69" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B69*$C$17/(1+$C$17),IF(O69="",0,B69*O69/(1+O69)))</f>
+        <v/>
+      </c>
+      <c r="U69" s="33">
+        <f>E69*Q69</f>
+        <v/>
+      </c>
+      <c r="V69" s="33">
+        <f>G69*Q69</f>
+        <v/>
+      </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="31" t="n">
@@ -14165,6 +14511,18 @@
         <f>ROUNDUP(A70/3,0)</f>
         <v/>
       </c>
+      <c r="T70" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B70*$C$17/(1+$C$17),IF(O70="",0,B70*O70/(1+O70)))</f>
+        <v/>
+      </c>
+      <c r="U70" s="33">
+        <f>E70*Q70</f>
+        <v/>
+      </c>
+      <c r="V70" s="33">
+        <f>G70*Q70</f>
+        <v/>
+      </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="31" t="n">
@@ -14242,6 +14600,18 @@
         <f>ROUNDUP(A71/3,0)</f>
         <v/>
       </c>
+      <c r="T71" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B71*$C$17/(1+$C$17),IF(O71="",0,B71*O71/(1+O71)))</f>
+        <v/>
+      </c>
+      <c r="U71" s="33">
+        <f>E71*Q71</f>
+        <v/>
+      </c>
+      <c r="V71" s="33">
+        <f>G71*Q71</f>
+        <v/>
+      </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="31" t="n">
@@ -14319,6 +14689,18 @@
         <f>ROUNDUP(A72/3,0)</f>
         <v/>
       </c>
+      <c r="T72" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B72*$C$17/(1+$C$17),IF(O72="",0,B72*O72/(1+O72)))</f>
+        <v/>
+      </c>
+      <c r="U72" s="33">
+        <f>E72*Q72</f>
+        <v/>
+      </c>
+      <c r="V72" s="33">
+        <f>G72*Q72</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="31" t="n">
@@ -14396,6 +14778,18 @@
         <f>ROUNDUP(A73/3,0)</f>
         <v/>
       </c>
+      <c r="T73" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B73*$C$17/(1+$C$17),IF(O73="",0,B73*O73/(1+O73)))</f>
+        <v/>
+      </c>
+      <c r="U73" s="33">
+        <f>E73*Q73</f>
+        <v/>
+      </c>
+      <c r="V73" s="33">
+        <f>G73*Q73</f>
+        <v/>
+      </c>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="31" t="n">
@@ -14473,6 +14867,18 @@
         <f>ROUNDUP(A74/3,0)</f>
         <v/>
       </c>
+      <c r="T74" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B74*$C$17/(1+$C$17),IF(O74="",0,B74*O74/(1+O74)))</f>
+        <v/>
+      </c>
+      <c r="U74" s="33">
+        <f>E74*Q74</f>
+        <v/>
+      </c>
+      <c r="V74" s="33">
+        <f>G74*Q74</f>
+        <v/>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="31" t="n">
@@ -14550,6 +14956,18 @@
         <f>ROUNDUP(A75/3,0)</f>
         <v/>
       </c>
+      <c r="T75" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B75*$C$17/(1+$C$17),IF(O75="",0,B75*O75/(1+O75)))</f>
+        <v/>
+      </c>
+      <c r="U75" s="33">
+        <f>E75*Q75</f>
+        <v/>
+      </c>
+      <c r="V75" s="33">
+        <f>G75*Q75</f>
+        <v/>
+      </c>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="31" t="n">
@@ -14627,6 +15045,18 @@
         <f>ROUNDUP(A76/3,0)</f>
         <v/>
       </c>
+      <c r="T76" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B76*$C$17/(1+$C$17),IF(O76="",0,B76*O76/(1+O76)))</f>
+        <v/>
+      </c>
+      <c r="U76" s="33">
+        <f>E76*Q76</f>
+        <v/>
+      </c>
+      <c r="V76" s="33">
+        <f>G76*Q76</f>
+        <v/>
+      </c>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="31" t="n">
@@ -14704,6 +15134,18 @@
         <f>ROUNDUP(A77/3,0)</f>
         <v/>
       </c>
+      <c r="T77" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B77*$C$17/(1+$C$17),IF(O77="",0,B77*O77/(1+O77)))</f>
+        <v/>
+      </c>
+      <c r="U77" s="33">
+        <f>E77*Q77</f>
+        <v/>
+      </c>
+      <c r="V77" s="33">
+        <f>G77*Q77</f>
+        <v/>
+      </c>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="31" t="n">
@@ -14781,6 +15223,18 @@
         <f>ROUNDUP(A78/3,0)</f>
         <v/>
       </c>
+      <c r="T78" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B78*$C$17/(1+$C$17),IF(O78="",0,B78*O78/(1+O78)))</f>
+        <v/>
+      </c>
+      <c r="U78" s="33">
+        <f>E78*Q78</f>
+        <v/>
+      </c>
+      <c r="V78" s="33">
+        <f>G78*Q78</f>
+        <v/>
+      </c>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="31" t="n">
@@ -14858,6 +15312,18 @@
         <f>ROUNDUP(A79/3,0)</f>
         <v/>
       </c>
+      <c r="T79" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B79*$C$17/(1+$C$17),IF(O79="",0,B79*O79/(1+O79)))</f>
+        <v/>
+      </c>
+      <c r="U79" s="33">
+        <f>E79*Q79</f>
+        <v/>
+      </c>
+      <c r="V79" s="33">
+        <f>G79*Q79</f>
+        <v/>
+      </c>
     </row>
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="31" t="n">
@@ -14935,6 +15401,18 @@
         <f>ROUNDUP(A80/3,0)</f>
         <v/>
       </c>
+      <c r="T80" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B80*$C$17/(1+$C$17),IF(O80="",0,B80*O80/(1+O80)))</f>
+        <v/>
+      </c>
+      <c r="U80" s="33">
+        <f>E80*Q80</f>
+        <v/>
+      </c>
+      <c r="V80" s="33">
+        <f>G80*Q80</f>
+        <v/>
+      </c>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="31" t="n">
@@ -15012,6 +15490,18 @@
         <f>ROUNDUP(A81/3,0)</f>
         <v/>
       </c>
+      <c r="T81" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B81*$C$17/(1+$C$17),IF(O81="",0,B81*O81/(1+O81)))</f>
+        <v/>
+      </c>
+      <c r="U81" s="33">
+        <f>E81*Q81</f>
+        <v/>
+      </c>
+      <c r="V81" s="33">
+        <f>G81*Q81</f>
+        <v/>
+      </c>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="31" t="n">
@@ -15089,6 +15579,18 @@
         <f>ROUNDUP(A82/3,0)</f>
         <v/>
       </c>
+      <c r="T82" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B82*$C$17/(1+$C$17),IF(O82="",0,B82*O82/(1+O82)))</f>
+        <v/>
+      </c>
+      <c r="U82" s="33">
+        <f>E82*Q82</f>
+        <v/>
+      </c>
+      <c r="V82" s="33">
+        <f>G82*Q82</f>
+        <v/>
+      </c>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="31" t="n">
@@ -15166,6 +15668,18 @@
         <f>ROUNDUP(A83/3,0)</f>
         <v/>
       </c>
+      <c r="T83" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B83*$C$17/(1+$C$17),IF(O83="",0,B83*O83/(1+O83)))</f>
+        <v/>
+      </c>
+      <c r="U83" s="33">
+        <f>E83*Q83</f>
+        <v/>
+      </c>
+      <c r="V83" s="33">
+        <f>G83*Q83</f>
+        <v/>
+      </c>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="31" t="n">
@@ -15243,6 +15757,18 @@
         <f>ROUNDUP(A84/3,0)</f>
         <v/>
       </c>
+      <c r="T84" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B84*$C$17/(1+$C$17),IF(O84="",0,B84*O84/(1+O84)))</f>
+        <v/>
+      </c>
+      <c r="U84" s="33">
+        <f>E84*Q84</f>
+        <v/>
+      </c>
+      <c r="V84" s="33">
+        <f>G84*Q84</f>
+        <v/>
+      </c>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="31" t="n">
@@ -15320,6 +15846,18 @@
         <f>ROUNDUP(A85/3,0)</f>
         <v/>
       </c>
+      <c r="T85" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B85*$C$17/(1+$C$17),IF(O85="",0,B85*O85/(1+O85)))</f>
+        <v/>
+      </c>
+      <c r="U85" s="33">
+        <f>E85*Q85</f>
+        <v/>
+      </c>
+      <c r="V85" s="33">
+        <f>G85*Q85</f>
+        <v/>
+      </c>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="31" t="n">
@@ -15397,6 +15935,18 @@
         <f>ROUNDUP(A86/3,0)</f>
         <v/>
       </c>
+      <c r="T86" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B86*$C$17/(1+$C$17),IF(O86="",0,B86*O86/(1+O86)))</f>
+        <v/>
+      </c>
+      <c r="U86" s="33">
+        <f>E86*Q86</f>
+        <v/>
+      </c>
+      <c r="V86" s="33">
+        <f>G86*Q86</f>
+        <v/>
+      </c>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="31" t="n">
@@ -15474,6 +16024,18 @@
         <f>ROUNDUP(A87/3,0)</f>
         <v/>
       </c>
+      <c r="T87" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B87*$C$17/(1+$C$17),IF(O87="",0,B87*O87/(1+O87)))</f>
+        <v/>
+      </c>
+      <c r="U87" s="33">
+        <f>E87*Q87</f>
+        <v/>
+      </c>
+      <c r="V87" s="33">
+        <f>G87*Q87</f>
+        <v/>
+      </c>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="31" t="n">
@@ -15551,6 +16113,18 @@
         <f>ROUNDUP(A88/3,0)</f>
         <v/>
       </c>
+      <c r="T88" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B88*$C$17/(1+$C$17),IF(O88="",0,B88*O88/(1+O88)))</f>
+        <v/>
+      </c>
+      <c r="U88" s="33">
+        <f>E88*Q88</f>
+        <v/>
+      </c>
+      <c r="V88" s="33">
+        <f>G88*Q88</f>
+        <v/>
+      </c>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="31" t="n">
@@ -15628,6 +16202,18 @@
         <f>ROUNDUP(A89/3,0)</f>
         <v/>
       </c>
+      <c r="T89" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B89*$C$17/(1+$C$17),IF(O89="",0,B89*O89/(1+O89)))</f>
+        <v/>
+      </c>
+      <c r="U89" s="33">
+        <f>E89*Q89</f>
+        <v/>
+      </c>
+      <c r="V89" s="33">
+        <f>G89*Q89</f>
+        <v/>
+      </c>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="31" t="n">
@@ -15705,6 +16291,18 @@
         <f>ROUNDUP(A90/3,0)</f>
         <v/>
       </c>
+      <c r="T90" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B90*$C$17/(1+$C$17),IF(O90="",0,B90*O90/(1+O90)))</f>
+        <v/>
+      </c>
+      <c r="U90" s="33">
+        <f>E90*Q90</f>
+        <v/>
+      </c>
+      <c r="V90" s="33">
+        <f>G90*Q90</f>
+        <v/>
+      </c>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="31" t="n">
@@ -15782,6 +16380,18 @@
         <f>ROUNDUP(A91/3,0)</f>
         <v/>
       </c>
+      <c r="T91" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B91*$C$17/(1+$C$17),IF(O91="",0,B91*O91/(1+O91)))</f>
+        <v/>
+      </c>
+      <c r="U91" s="33">
+        <f>E91*Q91</f>
+        <v/>
+      </c>
+      <c r="V91" s="33">
+        <f>G91*Q91</f>
+        <v/>
+      </c>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="31" t="n">
@@ -15859,6 +16469,18 @@
         <f>ROUNDUP(A92/3,0)</f>
         <v/>
       </c>
+      <c r="T92" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B92*$C$17/(1+$C$17),IF(O92="",0,B92*O92/(1+O92)))</f>
+        <v/>
+      </c>
+      <c r="U92" s="33">
+        <f>E92*Q92</f>
+        <v/>
+      </c>
+      <c r="V92" s="33">
+        <f>G92*Q92</f>
+        <v/>
+      </c>
     </row>
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="31" t="n">
@@ -15936,6 +16558,18 @@
         <f>ROUNDUP(A93/3,0)</f>
         <v/>
       </c>
+      <c r="T93" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B93*$C$17/(1+$C$17),IF(O93="",0,B93*O93/(1+O93)))</f>
+        <v/>
+      </c>
+      <c r="U93" s="33">
+        <f>E93*Q93</f>
+        <v/>
+      </c>
+      <c r="V93" s="33">
+        <f>G93*Q93</f>
+        <v/>
+      </c>
     </row>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="31" t="n">
@@ -16013,6 +16647,18 @@
         <f>ROUNDUP(A94/3,0)</f>
         <v/>
       </c>
+      <c r="T94" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B94*$C$17/(1+$C$17),IF(O94="",0,B94*O94/(1+O94)))</f>
+        <v/>
+      </c>
+      <c r="U94" s="33">
+        <f>E94*Q94</f>
+        <v/>
+      </c>
+      <c r="V94" s="33">
+        <f>G94*Q94</f>
+        <v/>
+      </c>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="31" t="n">
@@ -16090,6 +16736,18 @@
         <f>ROUNDUP(A95/3,0)</f>
         <v/>
       </c>
+      <c r="T95" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B95*$C$17/(1+$C$17),IF(O95="",0,B95*O95/(1+O95)))</f>
+        <v/>
+      </c>
+      <c r="U95" s="33">
+        <f>E95*Q95</f>
+        <v/>
+      </c>
+      <c r="V95" s="33">
+        <f>G95*Q95</f>
+        <v/>
+      </c>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="31" t="n">
@@ -16167,6 +16825,18 @@
         <f>ROUNDUP(A96/3,0)</f>
         <v/>
       </c>
+      <c r="T96" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B96*$C$17/(1+$C$17),IF(O96="",0,B96*O96/(1+O96)))</f>
+        <v/>
+      </c>
+      <c r="U96" s="33">
+        <f>E96*Q96</f>
+        <v/>
+      </c>
+      <c r="V96" s="33">
+        <f>G96*Q96</f>
+        <v/>
+      </c>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="31" t="n">
@@ -16244,6 +16914,18 @@
         <f>ROUNDUP(A97/3,0)</f>
         <v/>
       </c>
+      <c r="T97" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B97*$C$17/(1+$C$17),IF(O97="",0,B97*O97/(1+O97)))</f>
+        <v/>
+      </c>
+      <c r="U97" s="33">
+        <f>E97*Q97</f>
+        <v/>
+      </c>
+      <c r="V97" s="33">
+        <f>G97*Q97</f>
+        <v/>
+      </c>
     </row>
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="31" t="n">
@@ -16321,6 +17003,18 @@
         <f>ROUNDUP(A98/3,0)</f>
         <v/>
       </c>
+      <c r="T98" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B98*$C$17/(1+$C$17),IF(O98="",0,B98*O98/(1+O98)))</f>
+        <v/>
+      </c>
+      <c r="U98" s="33">
+        <f>E98*Q98</f>
+        <v/>
+      </c>
+      <c r="V98" s="33">
+        <f>G98*Q98</f>
+        <v/>
+      </c>
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="31" t="n">
@@ -16398,6 +17092,18 @@
         <f>ROUNDUP(A99/3,0)</f>
         <v/>
       </c>
+      <c r="T99" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B99*$C$17/(1+$C$17),IF(O99="",0,B99*O99/(1+O99)))</f>
+        <v/>
+      </c>
+      <c r="U99" s="33">
+        <f>E99*Q99</f>
+        <v/>
+      </c>
+      <c r="V99" s="33">
+        <f>G99*Q99</f>
+        <v/>
+      </c>
     </row>
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="31" t="n">
@@ -16475,6 +17181,18 @@
         <f>ROUNDUP(A100/3,0)</f>
         <v/>
       </c>
+      <c r="T100" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B100*$C$17/(1+$C$17),IF(O100="",0,B100*O100/(1+O100)))</f>
+        <v/>
+      </c>
+      <c r="U100" s="33">
+        <f>E100*Q100</f>
+        <v/>
+      </c>
+      <c r="V100" s="33">
+        <f>G100*Q100</f>
+        <v/>
+      </c>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="31" t="n">
@@ -16552,6 +17270,18 @@
         <f>ROUNDUP(A101/3,0)</f>
         <v/>
       </c>
+      <c r="T101" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B101*$C$17/(1+$C$17),IF(O101="",0,B101*O101/(1+O101)))</f>
+        <v/>
+      </c>
+      <c r="U101" s="33">
+        <f>E101*Q101</f>
+        <v/>
+      </c>
+      <c r="V101" s="33">
+        <f>G101*Q101</f>
+        <v/>
+      </c>
     </row>
     <row r="102" ht="30" customHeight="1" thickBot="1">
       <c r="A102" s="31" t="n">
@@ -16629,6 +17359,18 @@
         <f>ROUNDUP(A102/3,0)</f>
         <v/>
       </c>
+      <c r="T102" s="33">
+        <f>IF('Matriz Normativa &amp; Governança'!$C$8="Alíquota plena — sensibilidade",B102*$C$17/(1+$C$17),IF(O102="",0,B102*O102/(1+O102)))</f>
+        <v/>
+      </c>
+      <c r="U102" s="33">
+        <f>E102*Q102</f>
+        <v/>
+      </c>
+      <c r="V102" s="33">
+        <f>G102*Q102</f>
+        <v/>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" s="22" t="inlineStr">
@@ -16686,6 +17428,18 @@
       </c>
       <c r="R103" s="49">
         <f>SUM(R43:R102)</f>
+        <v/>
+      </c>
+      <c r="T103" s="49">
+        <f>SUM(T43:T102)</f>
+        <v/>
+      </c>
+      <c r="U103" s="49">
+        <f>SUM(U43:U102)</f>
+        <v/>
+      </c>
+      <c r="V103" s="49">
+        <f>SUM(V43:V102)</f>
         <v/>
       </c>
     </row>
@@ -16848,10 +17602,9 @@
           <t>DRE consolidada por cenário</t>
         </is>
       </c>
-      <c r="B6" s="134" t="inlineStr">
-        <is>
-          <t>Cenários: alíquota plena (regime de 2033 em diante) · Ativo: modo selecionado na Matriz</t>
-        </is>
+      <c r="B6" s="134">
+        <f>"Todas as colunas no modo: "&amp;'Matriz Normativa &amp; Governança'!$C$8&amp;" (selecionado na aba Matriz Normativa &amp; Governança)"</f>
+        <v/>
       </c>
       <c r="C6" s="9" t="n"/>
       <c r="D6" s="9" t="n"/>
@@ -16925,15 +17678,15 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>'Premissas &amp; Cenários'!$B$68</f>
+        <f>'Premissas &amp; Cenários'!B68+Fluxo_Incorporacao!$R$103</f>
         <v/>
       </c>
       <c r="C9" s="21">
-        <f>'Premissas &amp; Cenários'!$C$68</f>
+        <f>'Premissas &amp; Cenários'!C68+Fluxo_Incorporacao!$R$103</f>
         <v/>
       </c>
       <c r="D9" s="21">
-        <f>'Premissas &amp; Cenários'!$D$68</f>
+        <f>'Premissas &amp; Cenários'!D68+Fluxo_Incorporacao!$R$103</f>
         <v/>
       </c>
       <c r="E9" s="51">
@@ -18335,17 +19088,17 @@
     </row>
     <row r="64"/>
     <row r="65">
-      <c r="A65" s="119" t="inlineStr">
+      <c r="A65" s="120" t="inlineStr">
         <is>
           <t>Visão societária — permuta física (OCPC 01 / ICPC 31)</t>
         </is>
       </c>
-      <c r="B65" s="120" t="n"/>
-      <c r="C65" s="120" t="n"/>
-      <c r="D65" s="120" t="n"/>
-      <c r="E65" s="120" t="n"/>
-      <c r="F65" s="120" t="n"/>
-      <c r="G65" s="120" t="n"/>
+      <c r="B65" s="121" t="n"/>
+      <c r="C65" s="121" t="n"/>
+      <c r="D65" s="121" t="n"/>
+      <c r="E65" s="121" t="n"/>
+      <c r="F65" s="121" t="n"/>
+      <c r="G65" s="121" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="127" t="inlineStr">
@@ -18374,7 +19127,7 @@
         <f>E8</f>
         <v/>
       </c>
-      <c r="F67" s="121" t="inlineStr">
+      <c r="F67" s="119" t="inlineStr">
         <is>
           <t>Recebimentos das unidades vendidas.</t>
         </is>
@@ -18390,7 +19143,7 @@
         <f>'Premissas &amp; Cenários'!$G$56</f>
         <v/>
       </c>
-      <c r="F68" s="121" t="inlineStr">
+      <c r="F68" s="119" t="inlineStr">
         <is>
           <t>Unidades entregues ao permutante do terreno, reconhecidas pelo valor justo.</t>
         </is>
@@ -18406,7 +19159,7 @@
         <f>E67+E68</f>
         <v/>
       </c>
-      <c r="F69" s="121" t="inlineStr">
+      <c r="F69" s="119" t="inlineStr">
         <is>
           <t>Base para a margem contábil do empreendimento.</t>
         </is>
@@ -18422,7 +19175,7 @@
         <f>-E68</f>
         <v/>
       </c>
-      <c r="F70" s="121" t="inlineStr">
+      <c r="F70" s="119" t="inlineStr">
         <is>
           <t>Contrapartida da permuta no custo do imóvel.</t>
         </is>
@@ -18438,7 +19191,7 @@
         <f>E68+E70</f>
         <v/>
       </c>
-      <c r="F71" s="121" t="inlineStr">
+      <c r="F71" s="119" t="inlineStr">
         <is>
           <t>Nulo: a permuta não altera o lucro, só a receita e o custo.</t>
         </is>
@@ -18454,7 +19207,7 @@
         <f>IFERROR(E31/E69,0)</f>
         <v/>
       </c>
-      <c r="F72" s="121" t="inlineStr">
+      <c r="F72" s="119" t="inlineStr">
         <is>
           <t>Compara com a margem sobre o VGV tributável (linha 32).</t>
         </is>
@@ -18521,14 +19274,14 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="B3" s="121" t="inlineStr">
+      <c r="B3" s="119" t="inlineStr">
         <is>
           <t>Apuração por trimestre sobre a receita recebida, com a majoração da presunção sobre o excedente de R$ 1,25 mi por trimestre (saldo acumulado no ano).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="121" t="inlineStr">
+      <c r="B4" s="119" t="inlineStr">
         <is>
           <t>A permuta física sem torna não compõe a receita tributável. A majoração da CSLL vale a partir do 2º trimestre de 2026 (noventena).</t>
         </is>
@@ -19796,7 +20549,7 @@
         <f>D27-Fluxo_Incorporacao!$B$103</f>
         <v/>
       </c>
-      <c r="E28" s="121" t="inlineStr">
+      <c r="E28" s="119" t="inlineStr">
         <is>
           <t>Receita trimestral menos recebimentos do fluxo; deve ser zero.</t>
         </is>
@@ -19842,7 +20595,7 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="121" t="inlineStr">
+      <c r="A3" s="119" t="inlineStr">
         <is>
           <t>Carga tributária do cenário ativo por ano de recebimento. RET: opção efetivada antes de 01/01/2029, com patrimônio de afetação e sem créditos.</t>
         </is>
@@ -19929,18 +20682,18 @@
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="119" t="inlineStr">
+      <c r="A9" s="120" t="inlineStr">
         <is>
           <t>A) Regime regular — regime específico de imóveis (LC 214) + Lucro Presumido</t>
         </is>
       </c>
-      <c r="B9" s="120" t="n"/>
-      <c r="C9" s="120" t="n"/>
-      <c r="D9" s="120" t="n"/>
-      <c r="E9" s="120" t="n"/>
-      <c r="F9" s="120" t="n"/>
-      <c r="G9" s="120" t="n"/>
-      <c r="H9" s="120" t="n"/>
+      <c r="B9" s="121" t="n"/>
+      <c r="C9" s="121" t="n"/>
+      <c r="D9" s="121" t="n"/>
+      <c r="E9" s="121" t="n"/>
+      <c r="F9" s="121" t="n"/>
+      <c r="G9" s="121" t="n"/>
+      <c r="H9" s="121" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="123" t="inlineStr">
@@ -20115,18 +20868,18 @@
     </row>
     <row r="15"/>
     <row r="16">
-      <c r="A16" s="119" t="inlineStr">
+      <c r="A16" s="120" t="inlineStr">
         <is>
           <t>B) RET de transição — art. 485 da LC 214</t>
         </is>
       </c>
-      <c r="B16" s="120" t="n"/>
-      <c r="C16" s="120" t="n"/>
-      <c r="D16" s="120" t="n"/>
-      <c r="E16" s="120" t="n"/>
-      <c r="F16" s="120" t="n"/>
-      <c r="G16" s="120" t="n"/>
-      <c r="H16" s="120" t="n"/>
+      <c r="B16" s="121" t="n"/>
+      <c r="C16" s="121" t="n"/>
+      <c r="D16" s="121" t="n"/>
+      <c r="E16" s="121" t="n"/>
+      <c r="F16" s="121" t="n"/>
+      <c r="G16" s="121" t="n"/>
+      <c r="H16" s="121" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="123" t="inlineStr">
@@ -20331,35 +21084,35 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="121" t="inlineStr">
+      <c r="A27" s="119" t="inlineStr">
         <is>
           <t>• No RET a apropriação de créditos de IBS/CBS é vedada; por isso o custo de obra fica pelo valor bruto e só os tributos pagos são comparados.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="121" t="inlineStr">
+      <c r="A28" s="119" t="inlineStr">
         <is>
           <t>• O RET de transição exige patrimônio de afetação e opção efetivada antes de 01/01/2029; incorporação de interesse social: 1% (Premissas, B111).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="121" t="inlineStr">
+      <c r="A29" s="119" t="inlineStr">
         <is>
           <t>• O saldo credor do regime regular é ativo a ressarcir: só tem valor se houver ressarcimento ou uso em outras operações da SPE.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="121" t="inlineStr">
+      <c r="A30" s="119" t="inlineStr">
         <is>
           <t>• IRPJ/CSLL do regime regular pelo Lucro Presumido; Lucro Real não está modelado.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="121" t="inlineStr">
+      <c r="A31" s="119" t="inlineStr">
         <is>
           <t>• Tratamento da permuta física no RET (receita para fins do regime) deve ser validado antes do uso.</t>
         </is>
@@ -20538,7 +21291,7 @@
       </c>
       <c r="F10" s="27" t="inlineStr">
         <is>
-          <t>Débito sobre a base final à alíquota efetiva plena.</t>
+          <t>Débito sobre a base final, no modo de cálculo selecionado.</t>
         </is>
       </c>
     </row>
@@ -20735,7 +21488,7 @@
     <row r="22" ht="38.25" customHeight="1">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>Crédito de obra: a v3 aplicava 27% sobre todo o custo. A v4 separa folha (sem crédito), materiais (alíquota padrão) e serviços de construção (alíquota reduzida do art. 261), ponderando fornecedores do Simples.</t>
+          <t>Crédito de obra: a v3 aplicava 27% sobre todo o custo. A v4 separa materiais (alíquota padrão), serviços de construção terceirizados (alíquota reduzida do art. 261) e eventual folha própria de obra (sem crédito), ponderando fornecedores do Simples.</t>
         </is>
       </c>
     </row>
@@ -20843,56 +21596,56 @@
     </row>
     <row r="39"/>
     <row r="40">
-      <c r="A40" s="119" t="inlineStr">
+      <c r="A40" s="120" t="inlineStr">
         <is>
           <t>Alterações da versão 4</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="121" t="inlineStr">
+      <c r="A41" s="119" t="inlineStr">
         <is>
           <t>• Crédito de obra por composição de custo (Premissas, linhas 89 a 93).</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="121" t="inlineStr">
+      <c r="A42" s="119" t="inlineStr">
         <is>
           <t>• Crédito de despesas por categoria, com alíquota do fornecedor e parcela da base com crédito (linhas 97 a 102).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="121" t="inlineStr">
+      <c r="A43" s="119" t="inlineStr">
         <is>
           <t>• Débito e créditos por fora, com tributo embutido nos valores informados.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="121" t="inlineStr">
+      <c r="A44" s="119" t="inlineStr">
         <is>
           <t>• Tabela de transição 2026-2033 completa e usada como modo padrão; fator de crédito por ano e PIS/Cofins em 2026.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="121" t="inlineStr">
+      <c r="A45" s="119" t="inlineStr">
         <is>
           <t>• Nova aba IRPJ_CSLL Trimestral com a majoração da LC 224/2025 (parâmetro para desligar).</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="121" t="inlineStr">
+      <c r="A46" s="119" t="inlineStr">
         <is>
           <t>• Nova aba Comparativo RET (art. 485).</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="121" t="inlineStr">
+      <c r="A47" s="119" t="inlineStr">
         <is>
           <t>• Visão societária da permuta física na DRE (OCPC 01) e matriz normativa ampliada.</t>
         </is>

</xml_diff>